<commit_message>
feat: Catalogos completo (refresco cache, export, tipo de proveedor, contacto principal, clientes-que-lo-compran, import por pestana)
</commit_message>
<xml_diff>
--- a/Presentacioces productos.xlsx
+++ b/Presentacioces productos.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/juanes/Desktop/Plein Produce/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mickyarambula/Desktop/erp-plein/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{169D4E9C-85EA-584A-B2BD-88DAC85645CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC62B150-5571-7843-B88E-84CA57B75C93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8000" yWindow="2300" windowWidth="26840" windowHeight="15740" xr2:uid="{A51E0920-E9C2-584D-829E-2A3960C036C8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -119,21 +119,12 @@
     <t>14 bunch of 8 oz</t>
   </si>
   <si>
-    <t>~960 lb</t>
-  </si>
-  <si>
-    <t>~924 lb</t>
-  </si>
-  <si>
     <t>Total Peso</t>
   </si>
   <si>
     <t>Cajas por pallet</t>
   </si>
   <si>
-    <t>~800 lb</t>
-  </si>
-  <si>
     <t>6 ct</t>
   </si>
   <si>
@@ -312,6 +303,15 @@
   </si>
   <si>
     <t>Description</t>
+  </si>
+  <si>
+    <t>960 lb</t>
+  </si>
+  <si>
+    <t>924 lb</t>
+  </si>
+  <si>
+    <t>800 lb</t>
   </si>
 </sst>
 </file>
@@ -371,7 +371,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -425,11 +425,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -455,32 +470,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
@@ -496,6 +489,21 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -516,7 +524,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -832,7 +840,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95A782DC-57CF-8842-A55B-371750DCAD8C}">
-  <dimension ref="B3:T37"/>
+  <dimension ref="A3:T37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="11.5" bestFit="1" customWidth="1"/>
@@ -850,78 +858,79 @@
     <col min="17" max="17" width="14.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:20" x14ac:dyDescent="0.2">
-      <c r="B3" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="J3" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
-      <c r="O3" s="14"/>
-    </row>
-    <row r="4" spans="2:20" x14ac:dyDescent="0.2">
-      <c r="B4" s="6" t="s">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="B3" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="17"/>
+      <c r="F3" s="17"/>
+      <c r="G3" s="17"/>
+      <c r="J3" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="K3" s="16"/>
+      <c r="L3" s="16"/>
+      <c r="M3" s="16"/>
+      <c r="N3" s="16"/>
+      <c r="O3" s="16"/>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A4" s="19"/>
+      <c r="B4" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="E4" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="F4" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="G4" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="H4" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="F4" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="H4" s="8" t="s">
-        <v>88</v>
-      </c>
       <c r="I4" s="3"/>
-      <c r="J4" s="22" t="s">
+      <c r="J4" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="K4" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="L4" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="M4" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="K4" s="22" t="s">
+      <c r="N4" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="L4" s="22" t="s">
+      <c r="O4" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="M4" s="22" t="s">
+      <c r="P4" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="N4" s="22" t="s">
-        <v>86</v>
-      </c>
-      <c r="O4" s="22" t="s">
-        <v>87</v>
-      </c>
-      <c r="P4" s="23" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="5" spans="2:20" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
       <c r="B5" s="7" t="s">
         <v>2</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="E5" s="7">
         <v>48</v>
@@ -929,10 +938,10 @@
       <c r="F5" s="7">
         <v>22</v>
       </c>
-      <c r="G5" s="12">
+      <c r="G5" s="9">
         <v>1056</v>
       </c>
-      <c r="H5" s="12">
+      <c r="H5" s="9">
         <f>G5*35</f>
         <v>36960</v>
       </c>
@@ -941,10 +950,10 @@
         <v>2</v>
       </c>
       <c r="K5" s="7" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="L5" s="7" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="M5" s="7">
         <v>48</v>
@@ -952,7 +961,7 @@
       <c r="N5" s="7">
         <v>24</v>
       </c>
-      <c r="O5" s="12">
+      <c r="O5" s="9">
         <v>1152</v>
       </c>
       <c r="P5" s="7">
@@ -960,15 +969,15 @@
         <v>39168</v>
       </c>
     </row>
-    <row r="6" spans="2:20" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
       <c r="B6" s="7" t="s">
         <v>2</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="E6" s="7">
         <v>48</v>
@@ -976,25 +985,25 @@
       <c r="F6" s="7">
         <v>22</v>
       </c>
-      <c r="G6" s="12">
+      <c r="G6" s="9">
         <v>1056</v>
       </c>
-      <c r="H6" s="12">
+      <c r="H6" s="9">
         <f t="shared" ref="H6:H9" si="0">G6*35</f>
         <v>36960</v>
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="1"/>
     </row>
-    <row r="7" spans="2:20" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
       <c r="B7" s="7" t="s">
         <v>2</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="E7" s="7">
         <v>48</v>
@@ -1002,34 +1011,25 @@
       <c r="F7" s="7">
         <v>22</v>
       </c>
-      <c r="G7" s="12">
+      <c r="G7" s="9">
         <v>1056</v>
       </c>
-      <c r="H7" s="12">
+      <c r="H7" s="9">
         <f t="shared" si="0"/>
         <v>36960</v>
       </c>
       <c r="I7" s="2"/>
-      <c r="J7" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="K7" s="13"/>
-      <c r="L7" s="13"/>
-      <c r="M7" s="13"/>
-      <c r="N7" s="13"/>
-      <c r="O7" s="13"/>
-      <c r="P7" s="13"/>
       <c r="T7" s="2"/>
     </row>
-    <row r="8" spans="2:20" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
       <c r="B8" s="7" t="s">
         <v>2</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="E8" s="7">
         <v>48</v>
@@ -1037,49 +1037,34 @@
       <c r="F8" s="7">
         <v>22</v>
       </c>
-      <c r="G8" s="12">
+      <c r="G8" s="9">
         <v>1056</v>
       </c>
-      <c r="H8" s="12">
+      <c r="H8" s="9">
         <f t="shared" si="0"/>
         <v>36960</v>
       </c>
       <c r="I8" s="2"/>
-      <c r="J8" s="22" t="s">
-        <v>82</v>
-      </c>
-      <c r="K8" s="22" t="s">
-        <v>83</v>
-      </c>
-      <c r="L8" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="M8" s="22" t="s">
-        <v>84</v>
-      </c>
-      <c r="N8" s="22" t="s">
-        <v>85</v>
-      </c>
-      <c r="O8" s="22" t="s">
-        <v>86</v>
-      </c>
-      <c r="P8" s="22" t="s">
-        <v>87</v>
-      </c>
-      <c r="Q8" s="23" t="s">
-        <v>88</v>
-      </c>
+      <c r="J8" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="K8" s="17"/>
+      <c r="L8" s="17"/>
+      <c r="M8" s="17"/>
+      <c r="N8" s="17"/>
+      <c r="O8" s="17"/>
+      <c r="P8" s="17"/>
       <c r="T8" s="2"/>
     </row>
-    <row r="9" spans="2:20" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
       <c r="B9" s="7" t="s">
         <v>4</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="E9" s="7">
         <v>48</v>
@@ -1087,50 +1072,49 @@
       <c r="F9" s="7">
         <v>22</v>
       </c>
-      <c r="G9" s="12">
+      <c r="G9" s="9">
         <v>1056</v>
       </c>
-      <c r="H9" s="12">
+      <c r="H9" s="9">
         <f t="shared" si="0"/>
         <v>36960</v>
       </c>
       <c r="I9" s="2"/>
-      <c r="J9" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="K9" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="L9" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="M9" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="N9" s="7">
+      <c r="J9" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="K9" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="O9" s="7">
-        <v>26</v>
-      </c>
-      <c r="P9" s="12">
-        <v>2080</v>
-      </c>
-      <c r="Q9">
-        <f>P9*12</f>
-        <v>24960</v>
+      <c r="L9" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="M9" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="N9" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="O9" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="P9" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="Q9" s="15" t="s">
+        <v>85</v>
       </c>
       <c r="T9" s="2"/>
     </row>
-    <row r="10" spans="2:20" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
       <c r="B10" s="7" t="s">
         <v>4</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E10" s="7">
         <v>48</v>
@@ -1138,11 +1122,11 @@
       <c r="F10" s="7">
         <v>20</v>
       </c>
-      <c r="G10" s="12">
+      <c r="G10" s="9">
         <f>F10*E10</f>
         <v>960</v>
       </c>
-      <c r="H10" s="12">
+      <c r="H10" s="9">
         <f>G10*40</f>
         <v>38400</v>
       </c>
@@ -1151,30 +1135,30 @@
         <v>2</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="L10" s="7" t="s">
-        <v>3</v>
+        <v>47</v>
       </c>
       <c r="M10" s="7" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="N10" s="7">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O10" s="7">
         <v>26</v>
       </c>
-      <c r="P10" s="12">
-        <v>1560</v>
+      <c r="P10" s="9">
+        <v>2080</v>
       </c>
       <c r="Q10">
-        <f>P10*16</f>
+        <f>P10*12</f>
         <v>24960</v>
       </c>
       <c r="T10" s="2"/>
     </row>
-    <row r="11" spans="2:20" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
@@ -1186,30 +1170,30 @@
         <v>2</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="L11" s="7" t="s">
-        <v>53</v>
+        <v>3</v>
       </c>
       <c r="M11" s="7" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="N11" s="7">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="O11" s="7">
         <v>26</v>
       </c>
-      <c r="P11" s="12">
-        <v>1248</v>
+      <c r="P11" s="9">
+        <v>1560</v>
       </c>
       <c r="Q11">
-        <f>P11*20</f>
+        <f>P11*16</f>
         <v>24960</v>
       </c>
       <c r="T11" s="2"/>
     </row>
-    <row r="12" spans="2:20" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
@@ -1218,16 +1202,16 @@
       <c r="H12" s="1"/>
       <c r="I12" s="2"/>
       <c r="J12" s="7" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K12" s="7" t="s">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="L12" s="7" t="s">
-        <v>7</v>
+        <v>50</v>
       </c>
       <c r="M12" s="7" t="s">
-        <v>54</v>
+        <v>21</v>
       </c>
       <c r="N12" s="7">
         <v>48</v>
@@ -1235,16 +1219,16 @@
       <c r="O12" s="7">
         <v>26</v>
       </c>
-      <c r="P12" s="12">
+      <c r="P12" s="9">
         <v>1248</v>
       </c>
       <c r="Q12">
-        <f>P12*25</f>
-        <v>31200</v>
+        <f>P12*20</f>
+        <v>24960</v>
       </c>
       <c r="T12" s="2"/>
     </row>
-    <row r="13" spans="2:20" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.2">
       <c r="C13" s="1"/>
       <c r="D13" s="5"/>
       <c r="E13" s="1"/>
@@ -1256,45 +1240,45 @@
         <v>4</v>
       </c>
       <c r="K13" s="7" t="s">
-        <v>55</v>
+        <v>5</v>
       </c>
       <c r="L13" s="7" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="M13" s="7" t="s">
-        <v>8</v>
+        <v>51</v>
       </c>
       <c r="N13" s="7">
-        <v>80</v>
+        <v>48</v>
       </c>
       <c r="O13" s="7">
         <v>26</v>
       </c>
-      <c r="P13" s="12">
-        <v>2080</v>
+      <c r="P13" s="9">
+        <v>1248</v>
       </c>
       <c r="Q13">
-        <f>P13*10</f>
-        <v>20800</v>
+        <f>P13*25</f>
+        <v>31200</v>
       </c>
       <c r="T13" s="2"/>
     </row>
-    <row r="14" spans="2:20" x14ac:dyDescent="0.2">
-      <c r="B14" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="18"/>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="B14" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
       <c r="H14" s="1"/>
       <c r="I14" s="2"/>
       <c r="J14" s="7" t="s">
         <v>4</v>
       </c>
       <c r="K14" s="7" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="L14" s="7" t="s">
         <v>9</v>
@@ -1308,7 +1292,7 @@
       <c r="O14" s="7">
         <v>26</v>
       </c>
-      <c r="P14" s="12">
+      <c r="P14" s="9">
         <v>2080</v>
       </c>
       <c r="Q14">
@@ -1317,49 +1301,65 @@
       </c>
       <c r="T14" s="2"/>
     </row>
-    <row r="15" spans="2:20" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.2">
       <c r="B15" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="E15" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="F15" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="G15" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="H15" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="F15" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="H15" s="8" t="s">
-        <v>88</v>
-      </c>
       <c r="I15" s="2"/>
-      <c r="J15" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="K15" s="15"/>
-      <c r="L15" s="15"/>
-      <c r="M15" s="15"/>
-      <c r="N15" s="15"/>
-      <c r="O15" s="15"/>
-      <c r="P15" s="15"/>
+      <c r="J15" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="M15" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="N15" s="7">
+        <v>80</v>
+      </c>
+      <c r="O15" s="7">
+        <v>26</v>
+      </c>
+      <c r="P15" s="9">
+        <v>2080</v>
+      </c>
+      <c r="Q15">
+        <f>P15*10</f>
+        <v>20800</v>
+      </c>
       <c r="T15" s="4"/>
     </row>
-    <row r="16" spans="2:20" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.2">
       <c r="B16" s="8" t="s">
         <v>2</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="E16" s="8">
         <v>48</v>
@@ -1367,37 +1367,13 @@
       <c r="F16" s="8">
         <v>22</v>
       </c>
-      <c r="G16" s="17">
+      <c r="G16" s="10">
         <v>1056</v>
       </c>
       <c r="H16" s="8">
         <f>1056*36</f>
         <v>38016</v>
       </c>
-      <c r="J16" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="K16" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="L16" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="M16" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="N16" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="O16" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="P16" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q16" s="23" t="s">
-        <v>88</v>
-      </c>
       <c r="T16" s="2"/>
     </row>
     <row r="17" spans="2:17" x14ac:dyDescent="0.2">
@@ -1405,10 +1381,10 @@
         <v>2</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="E17" s="8">
         <v>48</v>
@@ -1416,49 +1392,32 @@
       <c r="F17" s="8">
         <v>22</v>
       </c>
-      <c r="G17" s="17">
+      <c r="G17" s="10">
         <v>1056</v>
       </c>
       <c r="H17" s="8">
         <f>G17*36</f>
         <v>38016</v>
       </c>
-      <c r="J17" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="K17" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="L17" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="M17" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="N17" s="7">
-        <v>120</v>
-      </c>
-      <c r="O17" s="7">
-        <v>26</v>
-      </c>
-      <c r="P17" s="12">
-        <f>O17*N17</f>
-        <v>3120</v>
-      </c>
-      <c r="Q17" s="7">
-        <f>P17*11</f>
-        <v>34320</v>
-      </c>
+      <c r="J17" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="K17" s="18"/>
+      <c r="L17" s="18"/>
+      <c r="M17" s="18"/>
+      <c r="N17" s="18"/>
+      <c r="O17" s="18"/>
+      <c r="P17" s="18"/>
     </row>
     <row r="18" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B18" s="8" t="s">
         <v>2</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="E18" s="8">
         <v>48</v>
@@ -1466,38 +1425,36 @@
       <c r="F18" s="8">
         <v>22</v>
       </c>
-      <c r="G18" s="17">
+      <c r="G18" s="10">
         <v>1056</v>
       </c>
       <c r="H18" s="8">
         <f t="shared" ref="H18:H20" si="1">G18*36</f>
         <v>38016</v>
       </c>
-      <c r="J18" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="K18" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="L18" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="M18" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="N18" s="7">
-        <v>120</v>
-      </c>
-      <c r="O18" s="7">
-        <v>26</v>
-      </c>
-      <c r="P18" s="12">
-        <f t="shared" ref="P18:P26" si="2">O18*N18</f>
-        <v>3120</v>
-      </c>
-      <c r="Q18" s="7">
-        <f>P18*12</f>
-        <v>37440</v>
+      <c r="J18" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="K18" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="L18" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="M18" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="N18" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O18" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="P18" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q18" s="15" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="19" spans="2:17" x14ac:dyDescent="0.2">
@@ -1505,10 +1462,10 @@
         <v>2</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="E19" s="8">
         <v>48</v>
@@ -1516,7 +1473,7 @@
       <c r="F19" s="8">
         <v>22</v>
       </c>
-      <c r="G19" s="17">
+      <c r="G19" s="10">
         <v>1056</v>
       </c>
       <c r="H19" s="8">
@@ -1527,27 +1484,27 @@
         <v>2</v>
       </c>
       <c r="K19" s="7" t="s">
-        <v>76</v>
+        <v>56</v>
       </c>
       <c r="L19" s="7" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="M19" s="7" t="s">
-        <v>18</v>
+        <v>57</v>
       </c>
       <c r="N19" s="7">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="O19" s="7">
         <v>26</v>
       </c>
-      <c r="P19" s="12">
-        <f t="shared" si="2"/>
-        <v>2080</v>
+      <c r="P19" s="9">
+        <f>O19*N19</f>
+        <v>3120</v>
       </c>
       <c r="Q19" s="7">
-        <f>P19*16</f>
-        <v>33280</v>
+        <f>P19*11</f>
+        <v>34320</v>
       </c>
     </row>
     <row r="20" spans="2:17" x14ac:dyDescent="0.2">
@@ -1555,10 +1512,10 @@
         <v>2</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="E20" s="8">
         <v>48</v>
@@ -1566,7 +1523,7 @@
       <c r="F20" s="8">
         <v>22</v>
       </c>
-      <c r="G20" s="17">
+      <c r="G20" s="10">
         <v>1056</v>
       </c>
       <c r="H20" s="8">
@@ -1577,13 +1534,13 @@
         <v>2</v>
       </c>
       <c r="K20" s="7" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="L20" s="7" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="M20" s="7" t="s">
-        <v>63</v>
+        <v>22</v>
       </c>
       <c r="N20" s="7">
         <v>120</v>
@@ -1591,13 +1548,13 @@
       <c r="O20" s="7">
         <v>26</v>
       </c>
-      <c r="P20" s="12">
-        <f t="shared" si="2"/>
+      <c r="P20" s="9">
+        <f t="shared" ref="P20:P28" si="2">O20*N20</f>
         <v>3120</v>
       </c>
       <c r="Q20" s="7">
-        <f>P20*9</f>
-        <v>28080</v>
+        <f>P20*12</f>
+        <v>37440</v>
       </c>
     </row>
     <row r="21" spans="2:17" x14ac:dyDescent="0.2">
@@ -1605,10 +1562,10 @@
         <v>4</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="E21" s="8">
         <v>48</v>
@@ -1616,7 +1573,7 @@
       <c r="F21" s="8">
         <v>22</v>
       </c>
-      <c r="G21" s="17">
+      <c r="G21" s="10">
         <v>1056</v>
       </c>
       <c r="H21" s="8">
@@ -1627,27 +1584,27 @@
         <v>2</v>
       </c>
       <c r="K21" s="7" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="L21" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="M21" s="7" t="s">
-        <v>65</v>
+        <v>18</v>
       </c>
       <c r="N21" s="7">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="O21" s="7">
         <v>26</v>
       </c>
-      <c r="P21" s="12">
+      <c r="P21" s="9">
         <f t="shared" si="2"/>
-        <v>2600</v>
+        <v>2080</v>
       </c>
       <c r="Q21" s="7">
-        <f>P21*14</f>
-        <v>36400</v>
+        <f>P21*16</f>
+        <v>33280</v>
       </c>
     </row>
     <row r="22" spans="2:17" x14ac:dyDescent="0.2">
@@ -1655,10 +1612,10 @@
         <v>4</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E22" s="8">
         <v>48</v>
@@ -1666,7 +1623,7 @@
       <c r="F22" s="8">
         <v>20</v>
       </c>
-      <c r="G22" s="17">
+      <c r="G22" s="10">
         <f>F22*E22</f>
         <v>960</v>
       </c>
@@ -1679,207 +1636,244 @@
         <v>2</v>
       </c>
       <c r="K22" s="7" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="L22" s="7" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="M22" s="7" t="s">
-        <v>21</v>
+        <v>60</v>
       </c>
       <c r="N22" s="7">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="O22" s="7">
         <v>26</v>
       </c>
-      <c r="P22" s="12">
+      <c r="P22" s="9">
+        <f t="shared" si="2"/>
+        <v>3120</v>
+      </c>
+      <c r="Q22" s="7">
+        <f>P22*9</f>
+        <v>28080</v>
+      </c>
+    </row>
+    <row r="23" spans="2:17" x14ac:dyDescent="0.2">
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="11"/>
+      <c r="G23" s="13"/>
+      <c r="J23" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="K23" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="L23" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="M23" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="N23" s="7">
+        <v>100</v>
+      </c>
+      <c r="O23" s="7">
+        <v>26</v>
+      </c>
+      <c r="P23" s="9">
+        <f t="shared" si="2"/>
+        <v>2600</v>
+      </c>
+      <c r="Q23" s="7">
+        <f>P23*14</f>
+        <v>36400</v>
+      </c>
+    </row>
+    <row r="24" spans="2:17" x14ac:dyDescent="0.2">
+      <c r="C24" s="1"/>
+      <c r="E24" s="1"/>
+      <c r="J24" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="K24" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="L24" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="M24" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="N24" s="7">
+        <v>50</v>
+      </c>
+      <c r="O24" s="7">
+        <v>26</v>
+      </c>
+      <c r="P24" s="9">
         <f t="shared" si="2"/>
         <v>1300</v>
       </c>
-      <c r="Q22" s="7">
-        <f>P22*20</f>
+      <c r="Q24" s="7">
+        <f>P24*20</f>
         <v>26000</v>
       </c>
     </row>
-    <row r="23" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="B23" s="19"/>
-      <c r="C23" s="19"/>
-      <c r="D23" s="19"/>
-      <c r="E23" s="20"/>
-      <c r="F23" s="19"/>
-      <c r="G23" s="21"/>
-      <c r="J23" s="7" t="s">
+    <row r="25" spans="2:17" x14ac:dyDescent="0.2">
+      <c r="C25" s="1"/>
+      <c r="J25" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="K23" s="7" t="s">
+      <c r="K25" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="L23" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="M23" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="N23" s="7">
+      <c r="L25" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="M25" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="N25" s="7">
         <v>120</v>
       </c>
-      <c r="O23" s="7">
+      <c r="O25" s="7">
         <v>26</v>
       </c>
-      <c r="P23" s="12">
+      <c r="P25" s="9">
         <f t="shared" si="2"/>
         <v>3120</v>
       </c>
-      <c r="Q23" s="7">
-        <f>P23*11</f>
+      <c r="Q25" s="7">
+        <f>P25*11</f>
         <v>34320</v>
       </c>
     </row>
-    <row r="24" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="B24" s="9"/>
-      <c r="C24" s="10"/>
-      <c r="E24" s="1"/>
-      <c r="J24" s="7" t="s">
+    <row r="26" spans="2:17" x14ac:dyDescent="0.2">
+      <c r="C26" s="1"/>
+      <c r="D26" s="5"/>
+      <c r="E26" s="1"/>
+      <c r="J26" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="K24" s="7" t="s">
+      <c r="K26" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="L24" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="M24" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="N24" s="7">
+      <c r="L26" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="M26" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="N26" s="7">
         <v>50</v>
       </c>
-      <c r="O24" s="7">
+      <c r="O26" s="7">
         <v>26</v>
       </c>
-      <c r="P24" s="12">
+      <c r="P26" s="9">
         <f t="shared" si="2"/>
         <v>1300</v>
       </c>
-      <c r="Q24" s="7">
-        <f>P24*28</f>
+      <c r="Q26" s="7">
+        <f>P26*28</f>
         <v>36400</v>
       </c>
     </row>
-    <row r="25" spans="2:17" s="9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="C25" s="10"/>
-      <c r="J25" s="7" t="s">
+    <row r="27" spans="2:17" x14ac:dyDescent="0.2">
+      <c r="C27" s="1"/>
+      <c r="D27" s="5"/>
+      <c r="E27" s="1"/>
+      <c r="J27" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="K25" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="L25" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="M25" s="7" t="s">
+      <c r="K27" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L27" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="M27" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="N25" s="7">
+      <c r="N27" s="7">
         <v>120</v>
       </c>
-      <c r="O25" s="7">
+      <c r="O27" s="7">
         <v>26</v>
       </c>
-      <c r="P25" s="12">
+      <c r="P27" s="9">
         <f t="shared" si="2"/>
         <v>3120</v>
       </c>
-      <c r="Q25" s="7">
-        <f>P25*5</f>
+      <c r="Q27" s="7">
+        <f>P27*5</f>
         <v>15600</v>
       </c>
     </row>
-    <row r="26" spans="2:17" s="9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="C26" s="10"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="10"/>
-      <c r="J26" s="7" t="s">
+    <row r="28" spans="2:17" x14ac:dyDescent="0.2">
+      <c r="C28" s="1"/>
+      <c r="D28" s="5"/>
+      <c r="E28" s="1"/>
+      <c r="J28" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="K26" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="L26" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="M26" s="7" t="s">
+      <c r="K28" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="L28" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="M28" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="N26" s="7">
+      <c r="N28" s="7">
         <v>120</v>
       </c>
-      <c r="O26" s="7">
+      <c r="O28" s="7">
         <v>26</v>
       </c>
-      <c r="P26" s="12">
+      <c r="P28" s="9">
         <f t="shared" si="2"/>
         <v>3120</v>
       </c>
-      <c r="Q26" s="7">
-        <f>P26*5</f>
+      <c r="Q28" s="7">
+        <f>P28*5</f>
         <v>15600</v>
       </c>
     </row>
-    <row r="27" spans="2:17" s="9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="C27" s="10"/>
-      <c r="D27" s="11"/>
-      <c r="E27" s="10"/>
-      <c r="J27" s="10"/>
-      <c r="K27" s="10"/>
-      <c r="L27" s="10"/>
-      <c r="M27" s="10"/>
-      <c r="N27" s="10"/>
-      <c r="O27" s="10"/>
-      <c r="P27" s="16"/>
-    </row>
-    <row r="28" spans="2:17" s="9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="C28" s="10"/>
-      <c r="D28" s="11"/>
-      <c r="E28" s="10"/>
-      <c r="J28" s="10"/>
-      <c r="K28" s="10"/>
-      <c r="L28" s="10"/>
-      <c r="M28" s="10"/>
-      <c r="N28" s="10"/>
-      <c r="O28" s="10"/>
-      <c r="P28" s="16"/>
-    </row>
-    <row r="29" spans="2:17" s="9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="C29" s="10"/>
-      <c r="D29" s="11"/>
-      <c r="E29" s="10"/>
-      <c r="J29" s="10"/>
-      <c r="K29" s="10"/>
-      <c r="L29" s="10"/>
-      <c r="M29" s="10"/>
-      <c r="N29" s="10"/>
-      <c r="O29" s="10"/>
-      <c r="P29" s="16"/>
-    </row>
-    <row r="30" spans="2:17" s="9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="C30" s="10"/>
-      <c r="D30" s="11"/>
-      <c r="E30" s="10"/>
+    <row r="29" spans="2:17" x14ac:dyDescent="0.2">
+      <c r="C29" s="1"/>
+      <c r="D29" s="5"/>
+      <c r="E29" s="1"/>
+      <c r="J29" s="1"/>
+      <c r="K29" s="1"/>
+      <c r="L29" s="1"/>
+      <c r="M29" s="1"/>
+      <c r="N29" s="1"/>
+      <c r="O29" s="1"/>
+      <c r="P29" s="2"/>
+    </row>
+    <row r="30" spans="2:17" x14ac:dyDescent="0.2">
+      <c r="C30" s="1"/>
+      <c r="D30" s="5"/>
+      <c r="E30" s="1"/>
     </row>
     <row r="31" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="B31" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="C31" s="14"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
-      <c r="F31" s="14"/>
-      <c r="G31" s="14"/>
-      <c r="H31" s="14"/>
-      <c r="I31" s="14"/>
-      <c r="J31" s="14"/>
+      <c r="B31" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="C31" s="16"/>
+      <c r="D31" s="16"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="16"/>
+      <c r="G31" s="16"/>
+      <c r="H31" s="16"/>
+      <c r="I31" s="16"/>
+      <c r="J31" s="16"/>
     </row>
     <row r="32" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B32" s="6" t="s">
@@ -1889,13 +1883,13 @@
         <v>1</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G32" s="6" t="s">
         <v>12</v>
@@ -1907,7 +1901,7 @@
         <v>14</v>
       </c>
       <c r="J32" s="6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="33" spans="2:10" x14ac:dyDescent="0.2">
@@ -1927,7 +1921,7 @@
         <v>80</v>
       </c>
       <c r="G33" s="7" t="s">
-        <v>26</v>
+        <v>88</v>
       </c>
       <c r="H33" s="7">
         <v>26</v>
@@ -1958,7 +1952,7 @@
         <v>132</v>
       </c>
       <c r="G34" s="7" t="s">
-        <v>27</v>
+        <v>89</v>
       </c>
       <c r="H34" s="7">
         <v>26</v>
@@ -1989,7 +1983,7 @@
         <v>50</v>
       </c>
       <c r="G35" s="7" t="s">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="H35" s="7">
         <v>24</v>
@@ -2011,7 +2005,7 @@
         <v>19</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>8</v>
@@ -2020,7 +2014,7 @@
         <v>80</v>
       </c>
       <c r="G36" s="7" t="s">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="H36" s="7">
         <v>24</v>
@@ -2042,7 +2036,7 @@
         <v>20</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E37" s="6" t="s">
         <v>21</v>
@@ -2051,7 +2045,7 @@
         <v>35</v>
       </c>
       <c r="G37" s="7" t="s">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="H37" s="7">
         <v>24</v>
@@ -2071,8 +2065,8 @@
     <mergeCell ref="B14:G14"/>
     <mergeCell ref="B3:G3"/>
     <mergeCell ref="J3:O3"/>
-    <mergeCell ref="J7:P7"/>
-    <mergeCell ref="J15:P15"/>
+    <mergeCell ref="J8:P8"/>
+    <mergeCell ref="J17:P17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>